<commit_message>
Refocus on coal: Mind ID flagship is coal (PTBA-style); replace nickel/bauxite with coal subsidiaries, DME gasification, HBA royalty, Tanjung Enim/Sumsel
</commit_message>
<xml_diff>
--- a/samples/04_Contoso_Minerals_Litigation_Cases.xlsx
+++ b/samples/04_Contoso_Minerals_Litigation_Cases.xlsx
@@ -565,12 +565,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gugatan Lingkungan — LSM Maju vs Contoso Bauxite</t>
+          <t>Gugatan Lingkungan — LSM Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — Mantan Karyawan Maju vs Contoso Gold</t>
+          <t>Wanprestasi Kontrak — Mantan Karyawan Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -853,12 +853,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gugatan Perdata Umum — LSM Berkah vs Contoso Bauxite</t>
+          <t>Gugatan Perdata Umum — LSM Berkah vs Contoso Coal</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — Warga Lestari vs Contoso Gold</t>
+          <t>Pembatalan SK IUP — Warga Lestari vs Contoso Coal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Arbitrase Komersial — CV Sejahtera vs Contoso Nickel</t>
+          <t>Arbitrase Komersial — CV Sejahtera vs Contoso Coal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Gugatan Lingkungan — CV Maju vs Contoso Bauxite</t>
+          <t>Gugatan Lingkungan — CV Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1333,12 +1333,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pidana Lingkungan — CV Nusantara vs Contoso Gold</t>
+          <t>Pidana Lingkungan — CV Nusantara vs Contoso Coal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — PT Berkah vs Contoso Bauxite</t>
+          <t>Wanprestasi Kontrak — PT Berkah vs Contoso Coal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Gugatan Perdata Umum — CV Lestari vs Contoso Nickel</t>
+          <t>Gugatan Perdata Umum — CV Lestari vs Contoso Coal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1717,12 +1717,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — Koperasi Berkah vs Contoso Tin</t>
+          <t>Pembatalan SK IUP — Koperasi Berkah vs Contoso DME</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1909,12 +1909,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sengketa Pajak — LSM Lestari vs Contoso Tin</t>
+          <t>Sengketa Pajak — LSM Lestari vs Contoso DME</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sengketa Hutan/KLHK — Warga Sejahtera vs Contoso Bauxite</t>
+          <t>Sengketa Hutan/KLHK — Warga Sejahtera vs Contoso Coal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2101,12 +2101,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gugatan Lingkungan — Koperasi Lestari vs Contoso Tin</t>
+          <t>Gugatan Lingkungan — Koperasi Lestari vs Contoso DME</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — Mantan Karyawan Maju vs Contoso Bauxite</t>
+          <t>Wanprestasi Kontrak — Mantan Karyawan Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2485,12 +2485,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gugatan Lingkungan — Koperasi Nusantara vs Contoso Tin</t>
+          <t>Gugatan Lingkungan — Koperasi Nusantara vs Contoso DME</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — Mantan Karyawan Sinar vs Contoso Gold</t>
+          <t>Wanprestasi Kontrak — Mantan Karyawan Sinar vs Contoso Coal</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2677,12 +2677,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sengketa Pajak — Warga Berkah vs Contoso Nickel</t>
+          <t>Sengketa Pajak — Warga Berkah vs Contoso Coal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2773,12 +2773,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sengketa Ketenagakerjaan — LSM Maju vs Contoso Gold</t>
+          <t>Sengketa Ketenagakerjaan — LSM Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gugatan Lingkungan — Koperasi Sejahtera vs Contoso Nickel</t>
+          <t>Gugatan Lingkungan — Koperasi Sejahtera vs Contoso Coal</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3157,12 +3157,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — Mantan Karyawan Sejahtera vs Contoso Nickel</t>
+          <t>Pembatalan SK IUP — Mantan Karyawan Sejahtera vs Contoso Coal</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3253,12 +3253,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sengketa Pertanahan — Warga Nusantara vs Contoso Tin</t>
+          <t>Sengketa Pertanahan — Warga Nusantara vs Contoso DME</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3445,12 +3445,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PT Contoso Nickel Sulawesi</t>
+          <t>PT Contoso Coal Sumsel</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — LSM Maju vs Contoso Nickel</t>
+          <t>Pembatalan SK IUP — LSM Maju vs Contoso Coal</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sengketa Pertanahan — PT Lestari vs Contoso Tin</t>
+          <t>Sengketa Pertanahan — PT Lestari vs Contoso DME</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3829,12 +3829,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — LSM Sejahtera vs Contoso Tin</t>
+          <t>Wanprestasi Kontrak — LSM Sejahtera vs Contoso DME</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4021,12 +4021,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — Mantan Karyawan Lestari vs Contoso Tin</t>
+          <t>Pembatalan SK IUP — Mantan Karyawan Lestari vs Contoso DME</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4309,12 +4309,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Arbitrase Komersial — LSM Lestari vs Contoso Bauxite</t>
+          <t>Arbitrase Komersial — LSM Lestari vs Contoso Coal</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4405,12 +4405,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pembatalan SK IUP — Warga Berkah vs Contoso Bauxite</t>
+          <t>Pembatalan SK IUP — Warga Berkah vs Contoso Coal</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4501,12 +4501,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wanprestasi Kontrak — Warga Berkah vs Contoso Tin</t>
+          <t>Wanprestasi Kontrak — Warga Berkah vs Contoso DME</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PT Contoso Gold Papua</t>
+          <t>PT Contoso Coal Jambi</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sengketa Pertanahan — PT Sinar vs Contoso Gold</t>
+          <t>Sengketa Pertanahan — PT Sinar vs Contoso Coal</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4885,12 +4885,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Sengketa Hutan/KLHK — CV Sinar vs Contoso Bauxite</t>
+          <t>Sengketa Hutan/KLHK — CV Sinar vs Contoso Coal</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4981,12 +4981,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Sengketa Hutan/KLHK — Warga Sejahtera vs Contoso Tin</t>
+          <t>Sengketa Hutan/KLHK — Warga Sejahtera vs Contoso DME</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5173,12 +5173,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PT Contoso Bauxite Kalimantan</t>
+          <t>PT Contoso Coal Kaltim</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sengketa Pajak — Koperasi Lestari vs Contoso Bauxite</t>
+          <t>Sengketa Pajak — Koperasi Lestari vs Contoso Coal</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5269,12 +5269,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PT Contoso Tin Bangka</t>
+          <t>PT Contoso DME Sumsel</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Pidana Lingkungan — PT Sejahtera vs Contoso Tin</t>
+          <t>Pidana Lingkungan — PT Sejahtera vs Contoso DME</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>